<commit_message>
feat: include overdue outstanding balance in Simple_Demo_Ledger.xlsx and dispatch instant email on upload
</commit_message>
<xml_diff>
--- a/public/Simple_Demo_Ledger.xlsx
+++ b/public/Simple_Demo_Ledger.xlsx
@@ -16,7 +16,7 @@
     <t>CLIENT CODE:</t>
   </si>
   <si>
-    <t>DEMO-101</t>
+    <t>OGL-909</t>
   </si>
   <si>
     <t/>
@@ -25,13 +25,13 @@
     <t>CLIENT NAME:</t>
   </si>
   <si>
-    <t>Apex Logistics Ltd</t>
+    <t>Olectra Greentech Ltd</t>
   </si>
   <si>
     <t>PERIOD:</t>
   </si>
   <si>
-    <t>01-Jan-2026 to 31-Aug-2026</t>
+    <t>01-May-2026 to 31-Aug-2026</t>
   </si>
   <si>
     <t>Date</t>
@@ -55,49 +55,49 @@
     <t>Amount</t>
   </si>
   <si>
-    <t>2026-07-15</t>
-  </si>
-  <si>
-    <t>INV-5001</t>
+    <t>2026-05-10</t>
+  </si>
+  <si>
+    <t>INV-8001</t>
   </si>
   <si>
     <t>invoice</t>
   </si>
   <si>
-    <t>John Doe</t>
-  </si>
-  <si>
-    <t>Freight Services</t>
-  </si>
-  <si>
-    <t>REF-99</t>
-  </si>
-  <si>
-    <t>2026-08-01</t>
-  </si>
-  <si>
-    <t>INV-5002</t>
-  </si>
-  <si>
-    <t>Jane Smith</t>
-  </si>
-  <si>
-    <t>Consulting Fee</t>
-  </si>
-  <si>
-    <t>REF-100</t>
-  </si>
-  <si>
-    <t>2026-08-20</t>
-  </si>
-  <si>
-    <t>RCT-1001</t>
+    <t>Rajesh Kumar</t>
+  </si>
+  <si>
+    <t>EV Bus Maintenance &amp; Parts</t>
+  </si>
+  <si>
+    <t>REF-801</t>
+  </si>
+  <si>
+    <t>2026-06-15</t>
+  </si>
+  <si>
+    <t>INV-8002</t>
+  </si>
+  <si>
+    <t>Priya Sharma</t>
+  </si>
+  <si>
+    <t>Fleet Telematics Subscription</t>
+  </si>
+  <si>
+    <t>REF-802</t>
+  </si>
+  <si>
+    <t>2026-07-20</t>
+  </si>
+  <si>
+    <t>RCT-4001</t>
   </si>
   <si>
     <t>receipt</t>
   </si>
   <si>
-    <t>Part Payment Received</t>
+    <t>Advance Part Payment</t>
   </si>
 </sst>
 </file>
@@ -554,7 +554,7 @@
         <v>19</v>
       </c>
       <c r="G5">
-        <v>150000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -577,7 +577,7 @@
         <v>24</v>
       </c>
       <c r="G6">
-        <v>250000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -600,7 +600,7 @@
         <v>19</v>
       </c>
       <c r="G7">
-        <v>-100000</v>
+        <v>-50000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: update Simple_Demo_Ledger.xlsx for Corporate Client (CLIENT_01) and update last_import_at timestamp
</commit_message>
<xml_diff>
--- a/public/Simple_Demo_Ledger.xlsx
+++ b/public/Simple_Demo_Ledger.xlsx
@@ -16,7 +16,7 @@
     <t>CLIENT CODE:</t>
   </si>
   <si>
-    <t>OGL-909</t>
+    <t>CLIENT_01</t>
   </si>
   <si>
     <t/>
@@ -25,7 +25,7 @@
     <t>CLIENT NAME:</t>
   </si>
   <si>
-    <t>Olectra Greentech Ltd</t>
+    <t>Corporate Client</t>
   </si>
   <si>
     <t>PERIOD:</t>
@@ -55,49 +55,49 @@
     <t>Amount</t>
   </si>
   <si>
-    <t>2026-05-10</t>
-  </si>
-  <si>
-    <t>INV-8001</t>
+    <t>2026-06-10</t>
+  </si>
+  <si>
+    <t>INV-9001</t>
   </si>
   <si>
     <t>invoice</t>
   </si>
   <si>
-    <t>Rajesh Kumar</t>
-  </si>
-  <si>
-    <t>EV Bus Maintenance &amp; Parts</t>
-  </si>
-  <si>
-    <t>REF-801</t>
-  </si>
-  <si>
-    <t>2026-06-15</t>
-  </si>
-  <si>
-    <t>INV-8002</t>
-  </si>
-  <si>
-    <t>Priya Sharma</t>
-  </si>
-  <si>
-    <t>Fleet Telematics Subscription</t>
-  </si>
-  <si>
-    <t>REF-802</t>
-  </si>
-  <si>
-    <t>2026-07-20</t>
-  </si>
-  <si>
-    <t>RCT-4001</t>
+    <t>Corporate User</t>
+  </si>
+  <si>
+    <t>Corporate Travel &amp; Part Billing</t>
+  </si>
+  <si>
+    <t>REF-901</t>
+  </si>
+  <si>
+    <t>2026-07-15</t>
+  </si>
+  <si>
+    <t>INV-9002</t>
+  </si>
+  <si>
+    <t>Executive User</t>
+  </si>
+  <si>
+    <t>Monthly Retainer Charge</t>
+  </si>
+  <si>
+    <t>REF-902</t>
+  </si>
+  <si>
+    <t>2026-08-01</t>
+  </si>
+  <si>
+    <t>RCT-5001</t>
   </si>
   <si>
     <t>receipt</t>
   </si>
   <si>
-    <t>Advance Part Payment</t>
+    <t>Partial Bank Transfer</t>
   </si>
 </sst>
 </file>
@@ -554,7 +554,7 @@
         <v>19</v>
       </c>
       <c r="G5">
-        <v>250000</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -577,7 +577,7 @@
         <v>24</v>
       </c>
       <c r="G6">
-        <v>180000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -600,7 +600,7 @@
         <v>19</v>
       </c>
       <c r="G7">
-        <v>-50000</v>
+        <v>-100000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>